<commit_message>
Fill matrix gaps: MLP, GNN LCPO weeks 2/4/6, GNN arch variants
Groups completed:
- Group 1: GNN LCPO weeks 2/4/6 (22 folds × 5 seeds each)
  → Row 18 cols F/G/H: 0.722±0.043 / 0.751±0.054 / 0.768±0.055
  → All 6 metric sheets updated
- Group 2: MLP all-features matched protocol (5 seeds, random+LCPO, all weeks)
  → Row 16 cols B-I across all 6 sheets (0.749→0.857 random, 0.734→0.829 LCPO)
- Group 3: GNN architectural variants (5 seeds each, week 8 random-student)
  → Row 21 with_enrollment_summaries: 0.884 ± 0.001
  → Row 22 enrollment_node:           0.883 ± 0.001
  → Row 23 edge_aware_mp:             0.884 ± 0.002
  → Row 25 temporal_features:         0.888 ± 0.002

Bug fixes:
- run_gnn_experiment.py: lcpo_summary.csv now appends (not overwrites) via
  _append_or_create_csv with dedup_keys=['week','fold_idx']
- run_gnn_experiment.py: random_student dedup keys now include 'condition'
  to prevent different conditions from silently overwriting each other
</commit_message>
<xml_diff>
--- a/AUROC_Results_Matrix_by_Dr_Guo.xlsx
+++ b/AUROC_Results_Matrix_by_Dr_Guo.xlsx
@@ -668,12 +668,8 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1136,21 +1132,21 @@
   <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -1167,7 +1163,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -1198,7 +1194,7 @@
       </c>
       <c r="O5" s="123" t="n"/>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="84">
       <c r="A6" s="123" t="n"/>
       <c r="B6" s="16" t="inlineStr">
         <is>
@@ -1271,7 +1267,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -1348,7 +1344,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="80" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -1417,7 +1413,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -1486,7 +1482,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="80" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -1555,7 +1551,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="81" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -1624,7 +1620,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="80" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -1701,7 +1697,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -1778,7 +1774,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="80" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -1855,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -1932,7 +1928,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="80" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
@@ -1940,42 +1936,42 @@
       </c>
       <c r="B16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.749 ± 0.004</t>
         </is>
       </c>
       <c r="C16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.810 ± 0.005</t>
         </is>
       </c>
       <c r="D16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.828 ± 0.003</t>
         </is>
       </c>
       <c r="E16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.857 ± 0.004</t>
         </is>
       </c>
       <c r="F16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.734 ± 0.048</t>
         </is>
       </c>
       <c r="G16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.781 ± 0.068</t>
         </is>
       </c>
       <c r="H16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.803 ± 0.080</t>
         </is>
       </c>
       <c r="I16" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.829 ± 0.084</t>
         </is>
       </c>
       <c r="J16" s="42" t="inlineStr">
@@ -2009,7 +2005,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="82" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -2086,7 +2082,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -2114,17 +2110,17 @@
       </c>
       <c r="F18" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.722 ± 0.043</t>
         </is>
       </c>
       <c r="G18" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.751 ± 0.054</t>
         </is>
       </c>
       <c r="H18" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.768 ± 0.055</t>
         </is>
       </c>
       <c r="I18" s="42" t="inlineStr">
@@ -2163,7 +2159,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -2240,7 +2236,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -2317,7 +2313,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -2340,7 +2336,7 @@
       </c>
       <c r="E21" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.884 ± 0.001</t>
         </is>
       </c>
       <c r="F21" s="37" t="inlineStr">
@@ -2394,7 +2390,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -2417,7 +2413,7 @@
       </c>
       <c r="E22" s="42" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.883 ± 0.001</t>
         </is>
       </c>
       <c r="F22" s="42" t="inlineStr">
@@ -2471,7 +2467,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -2494,7 +2490,7 @@
       </c>
       <c r="E23" s="37" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.884 ± 0.002</t>
         </is>
       </c>
       <c r="F23" s="37" t="inlineStr">
@@ -2548,7 +2544,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="83" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -2625,8 +2621,8 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="84" t="inlineStr">
+    <row r="25" ht="19" customHeight="1" s="84">
+      <c r="A25" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
         </is>
@@ -2648,7 +2644,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.888 ± 0.002</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2702,22 +2698,22 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="85" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="85" t="inlineStr">
         <is>
           <t>GCN</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="84" t="inlineStr">
+    <row r="28" ht="19" customHeight="1" s="84">
+      <c r="A28" t="inlineStr">
         <is>
           <t>R-GCN</t>
         </is>
@@ -2793,8 +2789,8 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="84" t="inlineStr">
+    <row r="29" ht="19" customHeight="1" s="84">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HGT</t>
         </is>
@@ -2870,8 +2866,8 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="84" t="inlineStr">
+    <row r="30" ht="19" customHeight="1" s="84">
+      <c r="A30" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
         </is>
@@ -2947,8 +2943,8 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="84" t="inlineStr">
+    <row r="31" ht="19" customHeight="1" s="84">
+      <c r="A31" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
         </is>
@@ -3024,8 +3020,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="84" t="inlineStr">
+    <row r="32" ht="19" customHeight="1" s="84">
+      <c r="A32" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
         </is>
@@ -3101,8 +3097,8 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="84" t="inlineStr">
+    <row r="33" ht="19" customHeight="1" s="84">
+      <c r="A33" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
         </is>
@@ -3178,8 +3174,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="84" t="inlineStr">
+    <row r="34" ht="19" customHeight="1" s="84">
+      <c r="A34" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
         </is>
@@ -3255,29 +3251,28 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" t="inlineStr">
         <is>
           <t>— = no verified result is currently available.  ± — = a supported mean exists, but its standard deviation is unavailable.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>
@@ -3311,21 +3306,21 @@
   <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -3342,7 +3337,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="55" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -3373,7 +3368,7 @@
       </c>
       <c r="O5" s="123" t="n"/>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="84">
       <c r="A6" s="123" t="n"/>
       <c r="B6" s="63" t="inlineStr">
         <is>
@@ -3446,7 +3441,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -3521,7 +3516,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="80" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -3574,7 +3569,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -3627,7 +3622,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="80" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -3680,7 +3675,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="81" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -3733,7 +3728,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="80" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -3808,7 +3803,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -3877,7 +3872,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="80" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -3946,7 +3941,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -4015,51 +4010,35 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="80" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
         </is>
       </c>
-      <c r="B16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B16" s="126" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="C16" s="126" t="n">
+        <v>0.852</v>
+      </c>
+      <c r="D16" s="126" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="E16" s="126" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="F16" s="126" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="G16" s="126" t="n">
+        <v>0.788</v>
+      </c>
+      <c r="H16" s="126" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I16" s="126" t="n">
+        <v>0.832</v>
       </c>
       <c r="J16" s="126" t="inlineStr">
         <is>
@@ -4092,7 +4071,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="82" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -4169,7 +4148,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -4187,20 +4166,14 @@
       <c r="E18" s="126" t="n">
         <v>0.881</v>
       </c>
-      <c r="F18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="126" t="n">
+        <v>0.732</v>
+      </c>
+      <c r="G18" s="126" t="n">
+        <v>0.772</v>
+      </c>
+      <c r="H18" s="126" t="n">
+        <v>0.793</v>
       </c>
       <c r="I18" s="126" t="n">
         <v>0.8100000000000001</v>
@@ -4232,7 +4205,7 @@
         <v>0.347</v>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -4301,7 +4274,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -4376,7 +4349,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -4397,10 +4370,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="128" t="n">
+        <v>0.913</v>
       </c>
       <c r="F21" s="128" t="inlineStr">
         <is>
@@ -4453,7 +4424,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -4474,10 +4445,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="126" t="n">
+        <v>0.913</v>
       </c>
       <c r="F22" s="126" t="inlineStr">
         <is>
@@ -4530,7 +4499,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -4551,10 +4520,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="128" t="n">
+        <v>0.912</v>
       </c>
       <c r="F23" s="128" t="inlineStr">
         <is>
@@ -4607,7 +4574,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="83" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -4684,8 +4651,8 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="84" t="inlineStr">
+    <row r="25" ht="19" customHeight="1" s="84">
+      <c r="A25" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
         </is>
@@ -4705,10 +4672,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E25" t="n">
+        <v>0.916</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -4761,22 +4726,22 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="85" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="85" t="inlineStr">
         <is>
           <t>GCN</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="84" t="inlineStr">
+    <row r="28" ht="19" customHeight="1" s="84">
+      <c r="A28" t="inlineStr">
         <is>
           <t>R-GCN</t>
         </is>
@@ -4852,8 +4817,8 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="84" t="inlineStr">
+    <row r="29" ht="19" customHeight="1" s="84">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HGT</t>
         </is>
@@ -4929,8 +4894,8 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="84" t="inlineStr">
+    <row r="30" ht="19" customHeight="1" s="84">
+      <c r="A30" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
         </is>
@@ -5004,8 +4969,8 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="84" t="inlineStr">
+    <row r="31" ht="19" customHeight="1" s="84">
+      <c r="A31" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
         </is>
@@ -5079,8 +5044,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="84" t="inlineStr">
+    <row r="32" ht="19" customHeight="1" s="84">
+      <c r="A32" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
         </is>
@@ -5154,8 +5119,8 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="84" t="inlineStr">
+    <row r="33" ht="19" customHeight="1" s="84">
+      <c r="A33" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
         </is>
@@ -5229,8 +5194,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="84" t="inlineStr">
+    <row r="34" ht="19" customHeight="1" s="84">
+      <c r="A34" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
         </is>
@@ -5304,29 +5269,28 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" t="inlineStr">
         <is>
           <t>— = no verified result is currently available. Planned rows remain unfilled until the matched protocol is completed.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>
@@ -5360,21 +5324,21 @@
   <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -5391,7 +5355,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="55" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -5422,7 +5386,7 @@
       </c>
       <c r="O5" s="123" t="n"/>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="84">
       <c r="A6" s="123" t="n"/>
       <c r="B6" s="63" t="inlineStr">
         <is>
@@ -5495,7 +5459,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -5570,7 +5534,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="80" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -5623,7 +5587,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -5676,7 +5640,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="80" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -5729,7 +5693,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="81" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -5782,7 +5746,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="80" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -5857,7 +5821,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -5926,7 +5890,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="80" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -5995,7 +5959,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -6064,51 +6028,35 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="80" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
         </is>
       </c>
-      <c r="B16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B16" s="126" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="C16" s="126" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="D16" s="126" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="E16" s="126" t="n">
+        <v>0.782</v>
+      </c>
+      <c r="F16" s="126" t="n">
+        <v>0.6820000000000001</v>
+      </c>
+      <c r="G16" s="126" t="n">
+        <v>0.694</v>
+      </c>
+      <c r="H16" s="126" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="I16" s="126" t="n">
+        <v>0.737</v>
       </c>
       <c r="J16" s="126" t="inlineStr">
         <is>
@@ -6141,7 +6089,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="82" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -6218,7 +6166,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -6236,20 +6184,14 @@
       <c r="E18" s="126" t="n">
         <v>0.76</v>
       </c>
-      <c r="F18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="126" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="G18" s="126" t="n">
+        <v>0.656</v>
+      </c>
+      <c r="H18" s="126" t="n">
+        <v>0.668</v>
       </c>
       <c r="I18" s="126" t="n">
         <v>0.678</v>
@@ -6281,7 +6223,7 @@
         <v>0.266</v>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -6350,7 +6292,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -6425,7 +6367,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -6446,10 +6388,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="128" t="n">
+        <v>0.8070000000000001</v>
       </c>
       <c r="F21" s="128" t="inlineStr">
         <is>
@@ -6502,7 +6442,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -6523,10 +6463,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="126" t="n">
+        <v>0.802</v>
       </c>
       <c r="F22" s="126" t="inlineStr">
         <is>
@@ -6579,7 +6517,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -6600,10 +6538,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="128" t="n">
+        <v>0.8070000000000001</v>
       </c>
       <c r="F23" s="128" t="inlineStr">
         <is>
@@ -6656,7 +6592,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="83" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -6733,8 +6669,8 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="84" t="inlineStr">
+    <row r="25" ht="19" customHeight="1" s="84">
+      <c r="A25" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
         </is>
@@ -6754,10 +6690,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E25" t="n">
+        <v>0.8110000000000001</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -6810,22 +6744,22 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="85" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="85" t="inlineStr">
         <is>
           <t>GCN</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="84" t="inlineStr">
+    <row r="28" ht="19" customHeight="1" s="84">
+      <c r="A28" t="inlineStr">
         <is>
           <t>R-GCN</t>
         </is>
@@ -6901,8 +6835,8 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="84" t="inlineStr">
+    <row r="29" ht="19" customHeight="1" s="84">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HGT</t>
         </is>
@@ -6978,8 +6912,8 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="84" t="inlineStr">
+    <row r="30" ht="19" customHeight="1" s="84">
+      <c r="A30" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
         </is>
@@ -7053,8 +6987,8 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="84" t="inlineStr">
+    <row r="31" ht="19" customHeight="1" s="84">
+      <c r="A31" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
         </is>
@@ -7128,8 +7062,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="84" t="inlineStr">
+    <row r="32" ht="19" customHeight="1" s="84">
+      <c r="A32" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
         </is>
@@ -7203,8 +7137,8 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="84" t="inlineStr">
+    <row r="33" ht="19" customHeight="1" s="84">
+      <c r="A33" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
         </is>
@@ -7278,8 +7212,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="84" t="inlineStr">
+    <row r="34" ht="19" customHeight="1" s="84">
+      <c r="A34" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
         </is>
@@ -7353,29 +7287,28 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" t="inlineStr">
         <is>
           <t>— = no verified result is currently available. Planned rows remain unfilled until the matched protocol is completed.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>
@@ -7409,21 +7342,21 @@
   <dimension ref="A2:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -7440,7 +7373,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="55" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -7471,7 +7404,7 @@
       </c>
       <c r="O5" s="123" t="n"/>
     </row>
-    <row r="6" ht="24" customHeight="1">
+    <row r="6" ht="24" customHeight="1" s="84">
       <c r="A6" s="123" t="n"/>
       <c r="B6" s="63" t="inlineStr">
         <is>
@@ -7544,7 +7477,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="79" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -7619,7 +7552,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="80" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -7672,7 +7605,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="81" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -7725,7 +7658,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="80" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -7778,7 +7711,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="81" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -7831,7 +7764,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="80" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -7906,7 +7839,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -7975,7 +7908,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="80" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -8044,7 +7977,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="81" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -8113,51 +8046,35 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="80" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
         </is>
       </c>
-      <c r="B16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B16" s="126" t="n">
+        <v>0.627</v>
+      </c>
+      <c r="C16" s="126" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="D16" s="126" t="n">
+        <v>0.712</v>
+      </c>
+      <c r="E16" s="126" t="n">
+        <v>0.759</v>
+      </c>
+      <c r="F16" s="126" t="n">
+        <v>0.609</v>
+      </c>
+      <c r="G16" s="126" t="n">
+        <v>0.664</v>
+      </c>
+      <c r="H16" s="126" t="n">
+        <v>0.6870000000000001</v>
+      </c>
+      <c r="I16" s="126" t="n">
+        <v>0.731</v>
       </c>
       <c r="J16" s="126" t="inlineStr">
         <is>
@@ -8190,7 +8107,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="82" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -8267,7 +8184,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -8285,20 +8202,14 @@
       <c r="E18" s="126" t="n">
         <v>0.751</v>
       </c>
-      <c r="F18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="126" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="G18" s="126" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="H18" s="126" t="n">
+        <v>0.65</v>
       </c>
       <c r="I18" s="126" t="n">
         <v>0.704</v>
@@ -8330,7 +8241,7 @@
         <v>0.504</v>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -8399,7 +8310,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -8474,7 +8385,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -8495,10 +8406,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="128" t="n">
+        <v>0.793</v>
       </c>
       <c r="F21" s="128" t="inlineStr">
         <is>
@@ -8551,7 +8460,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="80" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -8572,10 +8481,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="126" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="126" t="n">
+        <v>0.794</v>
       </c>
       <c r="F22" s="126" t="inlineStr">
         <is>
@@ -8628,7 +8535,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="81" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -8649,10 +8556,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="128" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="128" t="n">
+        <v>0.792</v>
       </c>
       <c r="F23" s="128" t="inlineStr">
         <is>
@@ -8705,7 +8610,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="83" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -8782,8 +8687,8 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="84" t="inlineStr">
+    <row r="25" ht="19" customHeight="1" s="84">
+      <c r="A25" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
         </is>
@@ -8803,10 +8708,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E25" t="n">
+        <v>0.797</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -8859,22 +8762,22 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="85" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="85" t="inlineStr">
         <is>
           <t>GCN</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
-      <c r="A28" s="84" t="inlineStr">
+    <row r="28" ht="19" customHeight="1" s="84">
+      <c r="A28" t="inlineStr">
         <is>
           <t>R-GCN</t>
         </is>
@@ -8950,8 +8853,8 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
-      <c r="A29" s="84" t="inlineStr">
+    <row r="29" ht="19" customHeight="1" s="84">
+      <c r="A29" t="inlineStr">
         <is>
           <t>HGT</t>
         </is>
@@ -9027,8 +8930,8 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
-      <c r="A30" s="84" t="inlineStr">
+    <row r="30" ht="19" customHeight="1" s="84">
+      <c r="A30" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
         </is>
@@ -9102,8 +9005,8 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
-      <c r="A31" s="84" t="inlineStr">
+    <row r="31" ht="19" customHeight="1" s="84">
+      <c r="A31" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
         </is>
@@ -9177,8 +9080,8 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
-      <c r="A32" s="84" t="inlineStr">
+    <row r="32" ht="19" customHeight="1" s="84">
+      <c r="A32" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
         </is>
@@ -9252,8 +9155,8 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
-      <c r="A33" s="84" t="inlineStr">
+    <row r="33" ht="19" customHeight="1" s="84">
+      <c r="A33" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
         </is>
@@ -9327,8 +9230,8 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
-      <c r="A34" s="84" t="inlineStr">
+    <row r="34" ht="19" customHeight="1" s="84">
+      <c r="A34" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
         </is>
@@ -9402,29 +9305,28 @@
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" t="inlineStr">
         <is>
           <t>— = no verified result is currently available. Planned rows remain unfilled until the matched protocol is completed.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>
@@ -9458,21 +9360,21 @@
   <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -9551,7 +9453,7 @@
       <c r="N4" s="19" t="n"/>
       <c r="O4" s="19" t="n"/>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="93" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -9588,7 +9490,7 @@
       </c>
       <c r="O5" s="135" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="22" customHeight="1" s="84">
       <c r="A6" s="98" t="n"/>
       <c r="B6" s="98" t="inlineStr">
         <is>
@@ -9661,7 +9563,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="109" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -9736,7 +9638,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="110" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -9789,7 +9691,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="110" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -9842,7 +9744,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="110" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -9895,7 +9797,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="110" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -9948,7 +9850,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="110" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -10023,7 +9925,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="110" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -10092,7 +9994,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="110" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -10161,7 +10063,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="110" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -10230,51 +10132,35 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="110" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
         </is>
       </c>
-      <c r="B16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B16" s="114" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="C16" s="114" t="n">
+        <v>0.6929999999999999</v>
+      </c>
+      <c r="D16" s="114" t="n">
+        <v>0.702</v>
+      </c>
+      <c r="E16" s="114" t="n">
+        <v>0.761</v>
+      </c>
+      <c r="F16" s="114" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="G16" s="114" t="n">
+        <v>0.634</v>
+      </c>
+      <c r="H16" s="114" t="n">
+        <v>0.661</v>
+      </c>
+      <c r="I16" s="114" t="n">
+        <v>0.701</v>
       </c>
       <c r="J16" s="114" t="inlineStr">
         <is>
@@ -10307,7 +10193,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="110" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -10384,7 +10270,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="118" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -10402,20 +10288,14 @@
       <c r="E18" s="119" t="n">
         <v>0.78</v>
       </c>
-      <c r="F18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="119" t="n">
+        <v>0.628</v>
+      </c>
+      <c r="G18" s="119" t="n">
+        <v>0.668</v>
+      </c>
+      <c r="H18" s="119" t="n">
+        <v>0.676</v>
       </c>
       <c r="I18" s="119" t="n">
         <v>0.772</v>
@@ -10447,7 +10327,7 @@
         <v>0.23</v>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -10516,7 +10396,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -10591,7 +10471,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -10612,10 +10492,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="114" t="n">
+        <v>0.803</v>
       </c>
       <c r="F21" s="114" t="inlineStr">
         <is>
@@ -10668,7 +10546,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -10689,10 +10567,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="114" t="n">
+        <v>0.8169999999999999</v>
       </c>
       <c r="F22" s="114" t="inlineStr">
         <is>
@@ -10745,7 +10621,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -10766,10 +10642,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="114" t="n">
+        <v>0.8</v>
       </c>
       <c r="F23" s="114" t="inlineStr">
         <is>
@@ -10822,7 +10696,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -10899,7 +10773,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
+    <row r="25" ht="19" customHeight="1" s="84">
       <c r="A25" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
@@ -10920,10 +10794,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E25" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E25" s="114" t="n">
+        <v>0.8070000000000001</v>
       </c>
       <c r="F25" s="114" t="inlineStr">
         <is>
@@ -10976,7 +10848,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
@@ -11053,7 +10925,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="110" t="inlineStr">
         <is>
           <t>GCN</t>
@@ -11130,7 +11002,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
+    <row r="28" ht="19" customHeight="1" s="84">
       <c r="A28" s="110" t="inlineStr">
         <is>
           <t>R-GCN</t>
@@ -11207,7 +11079,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
+    <row r="29" ht="19" customHeight="1" s="84">
       <c r="A29" s="110" t="inlineStr">
         <is>
           <t>HGT</t>
@@ -11284,7 +11156,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
+    <row r="30" ht="19" customHeight="1" s="84">
       <c r="A30" s="118" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
@@ -11359,7 +11231,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
+    <row r="31" ht="19" customHeight="1" s="84">
       <c r="A31" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
@@ -11434,7 +11306,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
+    <row r="32" ht="19" customHeight="1" s="84">
       <c r="A32" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
@@ -11509,7 +11381,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
+    <row r="33" ht="19" customHeight="1" s="84">
       <c r="A33" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
@@ -11584,7 +11456,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
+    <row r="34" ht="19" customHeight="1" s="84">
       <c r="A34" s="111" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
@@ -11676,7 +11548,7 @@
       <c r="N35" s="19" t="n"/>
       <c r="O35" s="19" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" s="122" t="inlineStr">
         <is>
           <t>— = no verified result is currently available. Planned rows remain unfilled until the matched protocol is completed.</t>
@@ -11697,7 +11569,7 @@
       <c r="N36" s="122" t="n"/>
       <c r="O36" s="122" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" s="122" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
@@ -11718,7 +11590,7 @@
       <c r="N37" s="122" t="n"/>
       <c r="O37" s="122" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" s="122" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
@@ -11739,7 +11611,7 @@
       <c r="N38" s="122" t="n"/>
       <c r="O38" s="122" t="n"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" s="122" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>
@@ -11781,21 +11653,21 @@
   <dimension ref="A1:O39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="46" customWidth="1" style="84" min="1" max="1"/>
+    <col width="13" customWidth="1" style="84" min="2" max="2"/>
+    <col width="13" customWidth="1" style="84" min="3" max="3"/>
+    <col width="13" customWidth="1" style="84" min="4" max="4"/>
+    <col width="13" customWidth="1" style="84" min="5" max="5"/>
+    <col width="13" customWidth="1" style="84" min="6" max="6"/>
+    <col width="13" customWidth="1" style="84" min="7" max="7"/>
+    <col width="13" customWidth="1" style="84" min="8" max="8"/>
+    <col width="13" customWidth="1" style="84" min="9" max="9"/>
+    <col width="13" customWidth="1" style="84" min="10" max="10"/>
+    <col width="13" customWidth="1" style="84" min="11" max="11"/>
+    <col width="13" customWidth="1" style="84" min="12" max="12"/>
+    <col width="13" customWidth="1" style="84" min="13" max="13"/>
+    <col width="13" customWidth="1" style="84" min="14" max="14"/>
+    <col width="13" customWidth="1" style="84" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -11874,7 +11746,7 @@
       <c r="N4" s="19" t="n"/>
       <c r="O4" s="19" t="n"/>
     </row>
-    <row r="5" ht="28" customHeight="1">
+    <row r="5" ht="28" customHeight="1" s="84">
       <c r="A5" s="93" t="inlineStr">
         <is>
           <t>Method or variant</t>
@@ -11911,7 +11783,7 @@
       </c>
       <c r="O5" s="135" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="22" customHeight="1" s="84">
       <c r="A6" s="98" t="n"/>
       <c r="B6" s="98" t="inlineStr">
         <is>
@@ -11984,7 +11856,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="19" customHeight="1">
+    <row r="7" ht="19" customHeight="1" s="84">
       <c r="A7" s="109" t="inlineStr">
         <is>
           <t>Majority</t>
@@ -12059,7 +11931,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
+    <row r="8" ht="19" customHeight="1" s="84">
       <c r="A8" s="110" t="inlineStr">
         <is>
           <t>Logistic regression</t>
@@ -12112,7 +11984,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="19" customHeight="1">
+    <row r="9" ht="19" customHeight="1" s="84">
       <c r="A9" s="110" t="inlineStr">
         <is>
           <t>Random forest</t>
@@ -12165,7 +12037,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="19" customHeight="1">
+    <row r="10" ht="19" customHeight="1" s="84">
       <c r="A10" s="110" t="inlineStr">
         <is>
           <t>XGBoost</t>
@@ -12218,7 +12090,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
+    <row r="11" ht="19" customHeight="1" s="84">
       <c r="A11" s="110" t="inlineStr">
         <is>
           <t>LightGBM — all features (historical protocol)</t>
@@ -12271,7 +12143,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
+    <row r="12" ht="19" customHeight="1" s="84">
       <c r="A12" s="110" t="inlineStr">
         <is>
           <t>LightGBM — all features (matched protocol)</t>
@@ -12346,7 +12218,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="19" customHeight="1">
+    <row r="13" ht="19" customHeight="1" s="84">
       <c r="A13" s="110" t="inlineStr">
         <is>
           <t>LightGBM — VLE only</t>
@@ -12415,7 +12287,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="19" customHeight="1">
+    <row r="14" ht="19" customHeight="1" s="84">
       <c r="A14" s="110" t="inlineStr">
         <is>
           <t>LightGBM — assessment only</t>
@@ -12484,7 +12356,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
+    <row r="15" ht="19" customHeight="1" s="84">
       <c r="A15" s="110" t="inlineStr">
         <is>
           <t>LightGBM — VLE + assessment</t>
@@ -12553,51 +12425,35 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
+    <row r="16" ht="19" customHeight="1" s="84">
       <c r="A16" s="110" t="inlineStr">
         <is>
           <t>MLP — all enrollment features</t>
         </is>
       </c>
-      <c r="B16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I16" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="B16" s="114" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="C16" s="114" t="n">
+        <v>0.8080000000000001</v>
+      </c>
+      <c r="D16" s="114" t="n">
+        <v>0.822</v>
+      </c>
+      <c r="E16" s="114" t="n">
+        <v>0.806</v>
+      </c>
+      <c r="F16" s="114" t="n">
+        <v>0.862</v>
+      </c>
+      <c r="G16" s="114" t="n">
+        <v>0.799</v>
+      </c>
+      <c r="H16" s="114" t="n">
+        <v>0.8139999999999999</v>
+      </c>
+      <c r="I16" s="114" t="n">
+        <v>0.8080000000000001</v>
       </c>
       <c r="J16" s="114" t="inlineStr">
         <is>
@@ -12630,7 +12486,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="19" customHeight="1">
+    <row r="17" ht="19" customHeight="1" s="84">
       <c r="A17" s="110" t="inlineStr">
         <is>
           <t>MLP — six behavioral summaries (no graph)</t>
@@ -12707,7 +12563,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="19" customHeight="1">
+    <row r="18" ht="19" customHeight="1" s="84">
       <c r="A18" s="118" t="inlineStr">
         <is>
           <t>GraphSAGE — base (weighted)</t>
@@ -12725,20 +12581,14 @@
       <c r="E18" s="119" t="n">
         <v>0.745</v>
       </c>
-      <c r="F18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H18" s="119" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F18" s="119" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="G18" s="119" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="H18" s="119" t="n">
+        <v>0.741</v>
       </c>
       <c r="I18" s="119" t="n">
         <v>0.65</v>
@@ -12770,7 +12620,7 @@
         <v>0.413</v>
       </c>
     </row>
-    <row r="19" ht="19" customHeight="1">
+    <row r="19" ht="19" customHeight="1" s="84">
       <c r="A19" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — base (unweighted)</t>
@@ -12839,7 +12689,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
+    <row r="20" ht="19" customHeight="1" s="84">
       <c r="A20" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + interaction attributes</t>
@@ -12914,7 +12764,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
+    <row r="21" ht="19" customHeight="1" s="84">
       <c r="A21" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + six enrollment summaries (matched protocol)</t>
@@ -12935,10 +12785,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E21" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E21" s="114" t="n">
+        <v>0.8129999999999999</v>
       </c>
       <c r="F21" s="114" t="inlineStr">
         <is>
@@ -12991,7 +12839,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
+    <row r="22" ht="19" customHeight="1" s="84">
       <c r="A22" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — enrollment-node representation</t>
@@ -13012,10 +12860,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E22" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E22" s="114" t="n">
+        <v>0.789</v>
       </c>
       <c r="F22" s="114" t="inlineStr">
         <is>
@@ -13068,7 +12914,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
+    <row r="23" ht="19" customHeight="1" s="84">
       <c r="A23" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE — edge-aware message passing</t>
@@ -13089,10 +12935,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E23" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E23" s="114" t="n">
+        <v>0.8139999999999999</v>
       </c>
       <c r="F23" s="114" t="inlineStr">
         <is>
@@ -13145,7 +12989,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="19" customHeight="1">
+    <row r="24" ht="19" customHeight="1" s="84">
       <c r="A24" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + explicit course-design features</t>
@@ -13222,7 +13066,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="19" customHeight="1">
+    <row r="25" ht="19" customHeight="1" s="84">
       <c r="A25" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + temporal behavior features</t>
@@ -13243,10 +13087,8 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E25" s="114" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E25" s="114" t="n">
+        <v>0.8159999999999999</v>
       </c>
       <c r="F25" s="114" t="inlineStr">
         <is>
@@ -13299,7 +13141,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
+    <row r="26" ht="19" customHeight="1" s="84">
       <c r="A26" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE + course-conditioned prediction</t>
@@ -13376,7 +13218,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="19" customHeight="1">
+    <row r="27" ht="19" customHeight="1" s="84">
       <c r="A27" s="110" t="inlineStr">
         <is>
           <t>GCN</t>
@@ -13453,7 +13295,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="19" customHeight="1">
+    <row r="28" ht="19" customHeight="1" s="84">
       <c r="A28" s="110" t="inlineStr">
         <is>
           <t>R-GCN</t>
@@ -13530,7 +13372,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="19" customHeight="1">
+    <row r="29" ht="19" customHeight="1" s="84">
       <c r="A29" s="110" t="inlineStr">
         <is>
           <t>HGT</t>
@@ -13607,7 +13449,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="19" customHeight="1">
+    <row r="30" ht="19" customHeight="1" s="84">
       <c r="A30" s="118" t="inlineStr">
         <is>
           <t>GraphSAGE − edge attributes</t>
@@ -13682,7 +13524,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="19" customHeight="1">
+    <row r="31" ht="19" customHeight="1" s="84">
       <c r="A31" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − temporal features</t>
@@ -13757,7 +13599,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="19" customHeight="1">
+    <row r="32" ht="19" customHeight="1" s="84">
       <c r="A32" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − course features</t>
@@ -13832,7 +13674,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="19" customHeight="1">
+    <row r="33" ht="19" customHeight="1" s="84">
       <c r="A33" s="110" t="inlineStr">
         <is>
           <t>GraphSAGE − VLE</t>
@@ -13907,7 +13749,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="19" customHeight="1">
+    <row r="34" ht="19" customHeight="1" s="84">
       <c r="A34" s="111" t="inlineStr">
         <is>
           <t>GraphSAGE − assessment</t>
@@ -13999,7 +13841,7 @@
       <c r="N35" s="19" t="n"/>
       <c r="O35" s="19" t="n"/>
     </row>
-    <row r="36" ht="18" customHeight="1">
+    <row r="36" ht="18" customHeight="1" s="84">
       <c r="A36" s="122" t="inlineStr">
         <is>
           <t>— = no verified result is currently available. Planned rows remain unfilled until the matched protocol is completed.</t>
@@ -14020,7 +13862,7 @@
       <c r="N36" s="122" t="n"/>
       <c r="O36" s="122" t="n"/>
     </row>
-    <row r="37" ht="18" customHeight="1">
+    <row r="37" ht="18" customHeight="1" s="84">
       <c r="A37" s="122" t="inlineStr">
         <is>
           <t>Matched comparisons must use identical labels, prediction cutoffs, enrollments, splits/folds, seeds, and training-only preprocessing.</t>
@@ -14041,7 +13883,7 @@
       <c r="N37" s="122" t="n"/>
       <c r="O37" s="122" t="n"/>
     </row>
-    <row r="38" ht="18" customHeight="1">
+    <row r="38" ht="18" customHeight="1" s="84">
       <c r="A38" s="122" t="inlineStr">
         <is>
           <t>Historical LightGBM and corrected GraphSAGE results are not directly comparable; use the matched-protocol rows for final claims.</t>
@@ -14062,7 +13904,7 @@
       <c r="N38" s="122" t="n"/>
       <c r="O38" s="122" t="n"/>
     </row>
-    <row r="39" ht="18" customHeight="1">
+    <row r="39" ht="18" customHeight="1" s="84">
       <c r="A39" s="122" t="inlineStr">
         <is>
           <t>Per-seed and per-fold repository CSV files remain the reproducible source of truth; update this matrix only from verified outputs.</t>

</xml_diff>

<commit_message>
Update matrix and report with new results
Matrix:
- Fix Future-Presentation cells (cols J-M rows 8-11) from raw float to '0.XXX' string format
- MLP, GNN LCPO, and GNN arch variants already committed in 0b365ca

Report:
- Updated headline KPIs: best GNN now 0.888 (temporal features), MLP 0.857
- New key finding: GNN variants surpass LightGBM on random-student split
- Added MLP baseline to all comparison tables (W2/4/6/8, random+LCPO)
- New GNN Variants section: enrollment-node/edge-aware/enrollment-summaries/temporal (0.883-0.888)
- GNN base model section now includes MLP as reference row
- LCPO multi-week table added (GNN 0.722→0.788 W2→W8 with LightGBM+MLP reference)
- Full comparison table updated with all 12 models
- 7 key findings revised to reflect GNN variants beating tabular baseline
- Next steps updated: LCPO of variants, multi-week ablations, combine top variants
</commit_message>
<xml_diff>
--- a/AUROC_Results_Matrix_by_Dr_Guo.xlsx
+++ b/AUROC_Results_Matrix_by_Dr_Guo.xlsx
@@ -1390,17 +1390,25 @@
           <t>0.804 ± 0.074</t>
         </is>
       </c>
-      <c r="J8" s="42" t="n">
-        <v>0.754</v>
-      </c>
-      <c r="K8" s="42" t="n">
-        <v>0.753</v>
-      </c>
-      <c r="L8" s="42" t="n">
-        <v>0.788</v>
-      </c>
-      <c r="M8" s="42" t="n">
-        <v>0.8090000000000001</v>
+      <c r="J8" s="42" t="inlineStr">
+        <is>
+          <t>0.754</t>
+        </is>
+      </c>
+      <c r="K8" s="42" t="inlineStr">
+        <is>
+          <t>0.753</t>
+        </is>
+      </c>
+      <c r="L8" s="42" t="inlineStr">
+        <is>
+          <t>0.788</t>
+        </is>
+      </c>
+      <c r="M8" s="42" t="inlineStr">
+        <is>
+          <t>0.809</t>
+        </is>
       </c>
       <c r="N8" s="42" t="inlineStr">
         <is>
@@ -1459,17 +1467,25 @@
           <t>0.826 ± 0.084</t>
         </is>
       </c>
-      <c r="J9" s="37" t="n">
-        <v>0.745</v>
-      </c>
-      <c r="K9" s="37" t="n">
-        <v>0.786</v>
-      </c>
-      <c r="L9" s="37" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="M9" s="37" t="n">
-        <v>0.843</v>
+      <c r="J9" s="37" t="inlineStr">
+        <is>
+          <t>0.745</t>
+        </is>
+      </c>
+      <c r="K9" s="37" t="inlineStr">
+        <is>
+          <t>0.786</t>
+        </is>
+      </c>
+      <c r="L9" s="37" t="inlineStr">
+        <is>
+          <t>0.810</t>
+        </is>
+      </c>
+      <c r="M9" s="37" t="inlineStr">
+        <is>
+          <t>0.843</t>
+        </is>
       </c>
       <c r="N9" s="37" t="inlineStr">
         <is>
@@ -1528,17 +1544,25 @@
           <t>0.825 ± 0.077</t>
         </is>
       </c>
-      <c r="J10" s="42" t="n">
-        <v>0.752</v>
-      </c>
-      <c r="K10" s="42" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="L10" s="42" t="n">
-        <v>0.797</v>
-      </c>
-      <c r="M10" s="42" t="n">
-        <v>0.824</v>
+      <c r="J10" s="42" t="inlineStr">
+        <is>
+          <t>0.752</t>
+        </is>
+      </c>
+      <c r="K10" s="42" t="inlineStr">
+        <is>
+          <t>0.780</t>
+        </is>
+      </c>
+      <c r="L10" s="42" t="inlineStr">
+        <is>
+          <t>0.797</t>
+        </is>
+      </c>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>0.824</t>
+        </is>
       </c>
       <c r="N10" s="42" t="inlineStr">
         <is>
@@ -1597,17 +1621,25 @@
           <t>0.835 ± 0.076</t>
         </is>
       </c>
-      <c r="J11" s="37" t="n">
-        <v>0.766</v>
-      </c>
-      <c r="K11" s="37" t="n">
-        <v>0.797</v>
-      </c>
-      <c r="L11" s="37" t="n">
-        <v>0.8129999999999999</v>
-      </c>
-      <c r="M11" s="37" t="n">
-        <v>0.84</v>
+      <c r="J11" s="37" t="inlineStr">
+        <is>
+          <t>0.766</t>
+        </is>
+      </c>
+      <c r="K11" s="37" t="inlineStr">
+        <is>
+          <t>0.797</t>
+        </is>
+      </c>
+      <c r="L11" s="37" t="inlineStr">
+        <is>
+          <t>0.813</t>
+        </is>
+      </c>
+      <c r="M11" s="37" t="inlineStr">
+        <is>
+          <t>0.840</t>
+        </is>
       </c>
       <c r="N11" s="37" t="inlineStr">
         <is>

</xml_diff>